<commit_message>
added data cleaning script
</commit_message>
<xml_diff>
--- a/Raw Data/Dictionaries/ef2014d.xlsx
+++ b/Raw Data/Dictionaries/ef2014d.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/27264b434cdc266c/Documents/STA 477/Final Project/Student Retention Time Series Analysis/Raw Data/Dictionaries/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_3888F0741F56A297C8DEF6C79EBBA4C6DA1F7A4F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14340" yWindow="-120" windowWidth="14955" windowHeight="11760"/>
+    <workbookView xWindow="996" yWindow="1290" windowWidth="14538" windowHeight="10314" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Introduction" sheetId="6" r:id="rId1"/>
@@ -425,7 +431,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.000"/>
   </numFmts>
@@ -554,14 +560,17 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
   </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -599,7 +608,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -671,7 +680,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -844,16 +853,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J19"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.1640625" defaultRowHeight="12.3" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="20.28515625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="14.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" width="20.27734375" style="2" customWidth="1"/>
+    <col min="2" max="2" width="14.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="16384" width="9.1640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="5" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" s="5" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="19" t="s">
         <v>97</v>
       </c>
@@ -867,7 +876,7 @@
       <c r="I1" s="19"/>
       <c r="J1" s="19"/>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" ht="12.6" x14ac:dyDescent="0.45">
       <c r="A2" s="21" t="s">
         <v>116</v>
       </c>
@@ -881,7 +890,7 @@
       <c r="I2" s="22"/>
       <c r="J2" s="22"/>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A3" s="7"/>
       <c r="B3" s="8"/>
       <c r="C3" s="8"/>
@@ -893,7 +902,7 @@
       <c r="I3" s="8"/>
       <c r="J3" s="8"/>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A4" s="3" t="s">
         <v>0</v>
       </c>
@@ -901,7 +910,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A5" s="2" t="s">
         <v>117</v>
       </c>
@@ -909,7 +918,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A6" s="3" t="s">
         <v>0</v>
       </c>
@@ -917,7 +926,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A7" s="2" t="s">
         <v>119</v>
       </c>
@@ -925,7 +934,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="195.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:10" ht="195.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A9" s="2" t="s">
         <v>1</v>
       </c>
@@ -941,7 +950,7 @@
       <c r="I9" s="20"/>
       <c r="J9" s="20"/>
     </row>
-    <row r="10" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B10" s="6"/>
       <c r="C10" s="6"/>
       <c r="D10" s="6"/>
@@ -952,7 +961,7 @@
       <c r="I10" s="6"/>
       <c r="J10" s="6"/>
     </row>
-    <row r="11" spans="1:10" ht="116.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:10" ht="116.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A11" s="2" t="s">
         <v>2</v>
       </c>
@@ -968,7 +977,7 @@
       <c r="I11" s="23"/>
       <c r="J11" s="23"/>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A13" s="19" t="s">
         <v>4</v>
       </c>
@@ -982,7 +991,7 @@
       <c r="I13" s="19"/>
       <c r="J13" s="19"/>
     </row>
-    <row r="15" spans="1:10" ht="77.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:10" ht="77.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A15" s="2" t="s">
         <v>5</v>
       </c>
@@ -998,7 +1007,7 @@
       <c r="I15" s="20"/>
       <c r="J15" s="20"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A16" s="2" t="s">
         <v>7</v>
       </c>
@@ -1014,7 +1023,7 @@
       <c r="I16" s="20"/>
       <c r="J16" s="20"/>
     </row>
-    <row r="17" spans="1:10" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:10" ht="27.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A17" s="2" t="s">
         <v>9</v>
       </c>
@@ -1030,7 +1039,7 @@
       <c r="I17" s="18"/>
       <c r="J17" s="18"/>
     </row>
-    <row r="18" spans="1:10" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:10" ht="27.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A18" s="2" t="s">
         <v>122</v>
       </c>
@@ -1046,7 +1055,7 @@
       <c r="I18" s="18"/>
       <c r="J18" s="18"/>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.4">
       <c r="A19" s="2" t="s">
         <v>10</v>
       </c>
@@ -1081,20 +1090,20 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G16"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.1640625" defaultRowHeight="12.3" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="9.140625" style="1"/>
-    <col min="2" max="2" width="12.140625" style="1" customWidth="1"/>
-    <col min="3" max="4" width="9.140625" style="1"/>
-    <col min="5" max="5" width="10.28515625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="14.140625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="73.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" width="9.1640625" style="1"/>
+    <col min="2" max="2" width="12.1640625" style="1" customWidth="1"/>
+    <col min="3" max="4" width="9.1640625" style="1"/>
+    <col min="5" max="5" width="10.27734375" style="1" customWidth="1"/>
+    <col min="6" max="6" width="14.1640625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="73.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="9.1640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="9" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" s="9" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A1" s="9" t="s">
         <v>11</v>
       </c>
@@ -1117,7 +1126,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -1140,7 +1149,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A3" s="1">
         <v>21001</v>
       </c>
@@ -1163,7 +1172,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A4" s="1">
         <v>21006</v>
       </c>
@@ -1186,7 +1195,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A5" s="1">
         <v>21011</v>
       </c>
@@ -1209,7 +1218,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A6" s="1">
         <v>21026</v>
       </c>
@@ -1232,7 +1241,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A7" s="1">
         <v>21031</v>
       </c>
@@ -1255,7 +1264,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A8" s="1">
         <v>21036</v>
       </c>
@@ -1278,7 +1287,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A9" s="1">
         <v>21041</v>
       </c>
@@ -1301,7 +1310,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A10" s="1">
         <v>21016</v>
       </c>
@@ -1324,7 +1333,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A11" s="1">
         <v>21046</v>
       </c>
@@ -1347,7 +1356,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A12" s="1">
         <v>21051</v>
       </c>
@@ -1370,7 +1379,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A13" s="1">
         <v>21056</v>
       </c>
@@ -1393,7 +1402,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A14" s="1">
         <v>21061</v>
       </c>
@@ -1416,7 +1425,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A15" s="1">
         <v>21021</v>
       </c>
@@ -1439,7 +1448,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A16" s="1">
         <v>24301</v>
       </c>
@@ -1469,17 +1478,17 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:C16"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="11.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.1640625" defaultRowHeight="10.199999999999999" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9.140625" style="15"/>
-    <col min="2" max="2" width="11.140625" style="15" customWidth="1"/>
-    <col min="3" max="3" width="144.85546875" style="15" customWidth="1"/>
-    <col min="4" max="16384" width="9.140625" style="16"/>
+    <col min="1" max="1" width="9.1640625" style="15"/>
+    <col min="2" max="2" width="11.1640625" style="15" customWidth="1"/>
+    <col min="3" max="3" width="144.83203125" style="15" customWidth="1"/>
+    <col min="4" max="16384" width="9.1640625" style="16"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="14" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" s="14" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="13" t="s">
         <v>11</v>
       </c>
@@ -1490,7 +1499,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="15">
         <v>1</v>
       </c>
@@ -1501,7 +1510,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="157.5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" ht="132.6" x14ac:dyDescent="0.35">
       <c r="A3" s="15">
         <v>21001</v>
       </c>
@@ -1512,7 +1521,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="90" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" ht="81.599999999999994" x14ac:dyDescent="0.35">
       <c r="A4" s="15">
         <v>21006</v>
       </c>
@@ -1523,7 +1532,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="15">
         <v>21011</v>
       </c>
@@ -1534,7 +1543,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="56.25" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" ht="51" x14ac:dyDescent="0.35">
       <c r="A6" s="15">
         <v>21026</v>
       </c>
@@ -1545,7 +1554,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="22.5" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" ht="20.399999999999999" x14ac:dyDescent="0.35">
       <c r="A7" s="15">
         <v>21031</v>
       </c>
@@ -1556,7 +1565,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="15">
         <v>21036</v>
       </c>
@@ -1567,7 +1576,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="15">
         <v>21041</v>
       </c>
@@ -1578,7 +1587,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="22.5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" s="15">
         <v>21016</v>
       </c>
@@ -1589,7 +1598,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="67.5" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:3" ht="51" x14ac:dyDescent="0.35">
       <c r="A11" s="15">
         <v>21046</v>
       </c>
@@ -1600,7 +1609,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="22.5" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:3" ht="20.399999999999999" x14ac:dyDescent="0.35">
       <c r="A12" s="15">
         <v>21051</v>
       </c>
@@ -1611,7 +1620,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" s="15">
         <v>21056</v>
       </c>
@@ -1622,7 +1631,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" s="15">
         <v>21061</v>
       </c>
@@ -1633,7 +1642,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="22.5" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" s="15">
         <v>21021</v>
       </c>
@@ -1644,7 +1653,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="146.25" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:3" ht="132.6" x14ac:dyDescent="0.35">
       <c r="A16" s="15">
         <v>24301</v>
       </c>
@@ -1662,21 +1671,21 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:H15"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.1640625" defaultRowHeight="12.3" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="9.140625" style="1"/>
-    <col min="2" max="2" width="13.5703125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="9.1640625" style="1"/>
+    <col min="2" max="2" width="13.5546875" style="1" customWidth="1"/>
     <col min="3" max="4" width="11" style="10" customWidth="1"/>
-    <col min="5" max="5" width="9.140625" style="17"/>
-    <col min="6" max="6" width="9.140625" style="1"/>
+    <col min="5" max="5" width="9.1640625" style="17"/>
+    <col min="6" max="6" width="9.1640625" style="1"/>
     <col min="7" max="7" width="11" style="10" customWidth="1"/>
-    <col min="8" max="8" width="73.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="16384" width="9.140625" style="1"/>
+    <col min="8" max="8" width="73.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="16384" width="9.1640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>11</v>
       </c>
@@ -1702,7 +1711,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A2" s="1">
         <v>21001</v>
       </c>
@@ -1728,7 +1737,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A3" s="1">
         <v>21006</v>
       </c>
@@ -1754,7 +1763,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A4" s="1">
         <v>21011</v>
       </c>
@@ -1780,7 +1789,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A5" s="1">
         <v>21026</v>
       </c>
@@ -1806,7 +1815,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A6" s="1">
         <v>21031</v>
       </c>
@@ -1832,7 +1841,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A7" s="1">
         <v>21036</v>
       </c>
@@ -1858,7 +1867,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A8" s="1">
         <v>21041</v>
       </c>
@@ -1884,7 +1893,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A9" s="1">
         <v>21016</v>
       </c>
@@ -1910,7 +1919,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A10" s="1">
         <v>21046</v>
       </c>
@@ -1936,7 +1945,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A11" s="1">
         <v>21051</v>
       </c>
@@ -1962,7 +1971,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A12" s="1">
         <v>21056</v>
       </c>
@@ -1988,7 +1997,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A13" s="1">
         <v>21061</v>
       </c>
@@ -2014,7 +2023,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A14" s="1">
         <v>21021</v>
       </c>
@@ -2040,7 +2049,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A15" s="1">
         <v>24301</v>
       </c>
@@ -2073,21 +2082,21 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:H15"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.1640625" defaultRowHeight="12.3" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="9.140625" style="1"/>
-    <col min="2" max="2" width="13.5703125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="9.1640625" style="1"/>
+    <col min="2" max="2" width="13.5546875" style="1" customWidth="1"/>
     <col min="3" max="4" width="11" style="10" customWidth="1"/>
-    <col min="5" max="5" width="9.140625" style="17"/>
-    <col min="6" max="6" width="9.140625" style="1"/>
+    <col min="5" max="5" width="9.1640625" style="17"/>
+    <col min="6" max="6" width="9.1640625" style="1"/>
     <col min="7" max="7" width="11" style="10" customWidth="1"/>
-    <col min="8" max="8" width="73.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="16384" width="9.140625" style="1"/>
+    <col min="8" max="8" width="73.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="16384" width="9.1640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>11</v>
       </c>
@@ -2113,7 +2122,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A2" s="1">
         <v>21001</v>
       </c>
@@ -2139,7 +2148,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A3" s="1">
         <v>21006</v>
       </c>
@@ -2165,7 +2174,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A4" s="1">
         <v>21011</v>
       </c>
@@ -2191,7 +2200,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A5" s="1">
         <v>21026</v>
       </c>
@@ -2217,7 +2226,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A6" s="1">
         <v>21031</v>
       </c>
@@ -2243,7 +2252,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A7" s="1">
         <v>21036</v>
       </c>
@@ -2269,7 +2278,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A8" s="1">
         <v>21041</v>
       </c>
@@ -2295,7 +2304,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A9" s="1">
         <v>21016</v>
       </c>
@@ -2321,7 +2330,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A10" s="1">
         <v>21046</v>
       </c>
@@ -2347,7 +2356,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A11" s="1">
         <v>21051</v>
       </c>
@@ -2373,7 +2382,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A12" s="1">
         <v>21056</v>
       </c>
@@ -2399,7 +2408,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A13" s="1">
         <v>21061</v>
       </c>
@@ -2425,7 +2434,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A14" s="1">
         <v>21021</v>
       </c>
@@ -2451,7 +2460,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.4">
       <c r="A15" s="1">
         <v>24301</v>
       </c>
@@ -2484,21 +2493,21 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:B15"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.1640625" defaultRowHeight="12.3" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="11.5703125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="36.5703125" style="1" customWidth="1"/>
-    <col min="3" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" width="11.5546875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="36.5546875" style="1" customWidth="1"/>
+    <col min="3" max="16384" width="9.1640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
         <v>70</v>
       </c>
@@ -2506,7 +2515,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A3" s="1" t="s">
         <v>72</v>
       </c>
@@ -2514,7 +2523,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A4" s="1" t="s">
         <v>74</v>
       </c>
@@ -2522,7 +2531,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A5" s="1" t="s">
         <v>76</v>
       </c>
@@ -2530,7 +2539,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A6" s="1" t="s">
         <v>78</v>
       </c>
@@ -2538,7 +2547,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A7" s="1" t="s">
         <v>80</v>
       </c>
@@ -2546,7 +2555,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A8" s="1" t="s">
         <v>82</v>
       </c>
@@ -2554,7 +2563,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A9" s="1" t="s">
         <v>84</v>
       </c>
@@ -2562,7 +2571,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A10" s="1" t="s">
         <v>86</v>
       </c>
@@ -2570,7 +2579,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A11" s="1" t="s">
         <v>88</v>
       </c>
@@ -2578,7 +2587,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A12" s="1" t="s">
         <v>19</v>
       </c>
@@ -2586,7 +2595,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A13" s="1" t="s">
         <v>91</v>
       </c>
@@ -2594,7 +2603,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A14" s="1" t="s">
         <v>93</v>
       </c>
@@ -2602,7 +2611,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A15" s="1" t="s">
         <v>95</v>
       </c>

</xml_diff>